<commit_message>
Sync updated venue workbook with 65 registered venues
</commit_message>
<xml_diff>
--- a/업체정보/업체정보_간편입력.xlsx
+++ b/업체정보/업체정보_간편입력.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="306">
   <si>
     <t>상호명</t>
   </si>
@@ -737,6 +737,398 @@
   </si>
   <si>
     <t>010-3443-0056</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울 강남구 강남대로62길 23 역삼빌딩 1층 </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>다슬음</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1484-3401</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 마포구 와우산로17길 19-17 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>맷집</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1384-7968</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 송파구 오금로11길 37 109호</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>호락호락</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1341-2682</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강서구 강서로5나길 16 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1325-2538</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>까치집</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>경기 남양주시 진접읍 해밀예당3로 7 2층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>술로맨스</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1329-7286</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 영등포구 도림로 445 102호</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>문래가온</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1336-1858</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>경기 안양시 만안구 장내로 101 지상1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>야간매점</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>010-6293-3439</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 학동로 342 SK허브블루상가 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>중앙실비</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1391-0320</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울 강남구 도산대로45길 10-2 1층 </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>트키</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1370-2654</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 학동로53길 19 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>타카이</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1455-0321</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 도산대로49길 6-7 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>더코너하우스</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1394-5990</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>테라스석 동반 가능</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>오제 오징어제육</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 도산대로27길 40 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1404-3971</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 논현로139길 12</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>모스가든</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1489-1988</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>룸 동반 가능</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 강남구 학동로 343 B1층 구월의소철</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1417-3212</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>구월의 소철</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울 강남구 학동로21길 6 </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>파퓰러커피</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1342-5064</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 동대문구 장한로6길 53 102호</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>동대문대하구이사계절집</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1370-4530</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 중구 다산로46길 36 2층, 3층, 4층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>신당육</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>02-6953-8816</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>소형견 가능</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>소형견 가능 리드줄 필수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울 중구 퇴계로 409-11 1층 </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>심세정</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1444-7579</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>별관, 테라스 가능</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 광진구 능동로 264 한사랑빌딩 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울돼지구이</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1336-1116</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울 중구 청계천로 360 나동 104호 </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wnch동묘(운치)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1330-8166</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>유모차, 케이지 필수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>케이지 필수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>전시회</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 동대문구 왕산로 131 2층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1394-8570</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>소형견, 테라스 가능</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 중구 다산로 232 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>오신돼지갈비</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1357-9288</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>유모차, 케이지 필수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 성북구 동소문로22길 64 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>금뚜껑</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1361-0997</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>테라스 가능</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">서울 중랑구 봉우재로43길 12 1층 </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>피자빌리지</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1448-1263</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 성북구 동소문로22길 57-16 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>메종 드 잠봉</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1403-0031</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 성북구 고려대로7길 48 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>운치</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1475-4644</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 중구 퇴계로81길 10 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>누리담</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1386-3922</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>유모차, 케이지 필수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 중구 퇴계로 461 1층 101호</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>보메청담</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>02-2233-0937</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울 성북구 고려대로1길 69 1층</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>펫터니아 하우스</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0507-1334-2014</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -3365,641 +3757,1535 @@
       </c>
     </row>
     <row r="38" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="15"/>
-      <c r="I38" s="15"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="16"/>
-      <c r="O38" s="19"/>
+      <c r="A38" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="D38" s="15">
+        <v>0</v>
+      </c>
+      <c r="E38" s="15">
+        <v>0</v>
+      </c>
+      <c r="F38" s="15">
+        <v>0</v>
+      </c>
+      <c r="G38" s="15">
+        <v>0</v>
+      </c>
+      <c r="H38" s="15">
+        <v>1</v>
+      </c>
+      <c r="I38" s="15">
+        <v>0</v>
+      </c>
+      <c r="J38" s="16">
+        <v>0</v>
+      </c>
+      <c r="K38" s="16">
+        <v>1</v>
+      </c>
+      <c r="L38" s="16">
+        <v>0</v>
+      </c>
+      <c r="M38" s="16">
+        <v>0</v>
+      </c>
+      <c r="N38" s="16">
+        <v>0</v>
+      </c>
+      <c r="O38" s="19">
+        <v>0</v>
+      </c>
       <c r="P38" s="14"/>
       <c r="Q38" s="17" t="str">
         <f>IF(LEN(TRIM(B38))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B38),FIND(" ",TRIM(B38)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B38),FIND(" ",TRIM(B38)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="39" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A39" s="14"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
-      <c r="F39" s="15"/>
-      <c r="G39" s="15"/>
-      <c r="H39" s="15"/>
-      <c r="I39" s="15"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="16"/>
-      <c r="O39" s="19"/>
+      <c r="A39" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="D39" s="15">
+        <v>0</v>
+      </c>
+      <c r="E39" s="15">
+        <v>0</v>
+      </c>
+      <c r="F39" s="15">
+        <v>0</v>
+      </c>
+      <c r="G39" s="15">
+        <v>0</v>
+      </c>
+      <c r="H39" s="15">
+        <v>1</v>
+      </c>
+      <c r="I39" s="15">
+        <v>0</v>
+      </c>
+      <c r="J39" s="16">
+        <v>0</v>
+      </c>
+      <c r="K39" s="16">
+        <v>1</v>
+      </c>
+      <c r="L39" s="16">
+        <v>0</v>
+      </c>
+      <c r="M39" s="16">
+        <v>0</v>
+      </c>
+      <c r="N39" s="16">
+        <v>0</v>
+      </c>
+      <c r="O39" s="19">
+        <v>0</v>
+      </c>
       <c r="P39" s="14"/>
       <c r="Q39" s="17" t="str">
         <f>IF(LEN(TRIM(B39))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B39),FIND(" ",TRIM(B39)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B39),FIND(" ",TRIM(B39)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="40" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A40" s="14"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="15"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="15"/>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="16"/>
-      <c r="O40" s="19"/>
+      <c r="A40" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="D40" s="15">
+        <v>0</v>
+      </c>
+      <c r="E40" s="15">
+        <v>0</v>
+      </c>
+      <c r="F40" s="15">
+        <v>0</v>
+      </c>
+      <c r="G40" s="15">
+        <v>0</v>
+      </c>
+      <c r="H40" s="15">
+        <v>1</v>
+      </c>
+      <c r="I40" s="15">
+        <v>0</v>
+      </c>
+      <c r="J40" s="16">
+        <v>0</v>
+      </c>
+      <c r="K40" s="16">
+        <v>1</v>
+      </c>
+      <c r="L40" s="16">
+        <v>0</v>
+      </c>
+      <c r="M40" s="16">
+        <v>0</v>
+      </c>
+      <c r="N40" s="16">
+        <v>0</v>
+      </c>
+      <c r="O40" s="19">
+        <v>0</v>
+      </c>
       <c r="P40" s="14"/>
       <c r="Q40" s="17" t="str">
         <f>IF(LEN(TRIM(B40))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B40),FIND(" ",TRIM(B40)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B40),FIND(" ",TRIM(B40)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="41" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15"/>
-      <c r="J41" s="16"/>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="16"/>
-      <c r="O41" s="19"/>
+      <c r="A41" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="D41" s="15">
+        <v>0</v>
+      </c>
+      <c r="E41" s="15">
+        <v>0</v>
+      </c>
+      <c r="F41" s="15">
+        <v>0</v>
+      </c>
+      <c r="G41" s="15">
+        <v>0</v>
+      </c>
+      <c r="H41" s="15">
+        <v>1</v>
+      </c>
+      <c r="I41" s="15">
+        <v>0</v>
+      </c>
+      <c r="J41" s="16">
+        <v>1</v>
+      </c>
+      <c r="K41" s="16">
+        <v>1</v>
+      </c>
+      <c r="L41" s="16">
+        <v>0</v>
+      </c>
+      <c r="M41" s="16">
+        <v>0</v>
+      </c>
+      <c r="N41" s="16">
+        <v>0</v>
+      </c>
+      <c r="O41" s="19">
+        <v>0</v>
+      </c>
       <c r="P41" s="14"/>
       <c r="Q41" s="17" t="str">
         <f>IF(LEN(TRIM(B41))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B41),FIND(" ",TRIM(B41)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B41),FIND(" ",TRIM(B41)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A42" s="14"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="15"/>
-      <c r="I42" s="15"/>
-      <c r="J42" s="16"/>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="16"/>
-      <c r="O42" s="19"/>
+      <c r="A42" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D42" s="15">
+        <v>0</v>
+      </c>
+      <c r="E42" s="15">
+        <v>0</v>
+      </c>
+      <c r="F42" s="15">
+        <v>0</v>
+      </c>
+      <c r="G42" s="15">
+        <v>0</v>
+      </c>
+      <c r="H42" s="15">
+        <v>1</v>
+      </c>
+      <c r="I42" s="15">
+        <v>0</v>
+      </c>
+      <c r="J42" s="16">
+        <v>1</v>
+      </c>
+      <c r="K42" s="16">
+        <v>1</v>
+      </c>
+      <c r="L42" s="16">
+        <v>1</v>
+      </c>
+      <c r="M42" s="16">
+        <v>0</v>
+      </c>
+      <c r="N42" s="16">
+        <v>0</v>
+      </c>
+      <c r="O42" s="19">
+        <v>0</v>
+      </c>
       <c r="P42" s="14"/>
       <c r="Q42" s="17" t="str">
         <f>IF(LEN(TRIM(B42))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B42),FIND(" ",TRIM(B42)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B42),FIND(" ",TRIM(B42)&amp;" ")-1)))</f>
-        <v/>
+        <v>경기</v>
       </c>
     </row>
     <row r="43" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A43" s="14"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15"/>
-      <c r="J43" s="16"/>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="16"/>
-      <c r="O43" s="19"/>
+      <c r="A43" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="D43" s="15">
+        <v>0</v>
+      </c>
+      <c r="E43" s="15">
+        <v>0</v>
+      </c>
+      <c r="F43" s="15">
+        <v>0</v>
+      </c>
+      <c r="G43" s="15">
+        <v>0</v>
+      </c>
+      <c r="H43" s="15">
+        <v>1</v>
+      </c>
+      <c r="I43" s="15">
+        <v>0</v>
+      </c>
+      <c r="J43" s="16">
+        <v>1</v>
+      </c>
+      <c r="K43" s="16">
+        <v>1</v>
+      </c>
+      <c r="L43" s="16">
+        <v>0</v>
+      </c>
+      <c r="M43" s="16">
+        <v>0</v>
+      </c>
+      <c r="N43" s="16">
+        <v>0</v>
+      </c>
+      <c r="O43" s="19">
+        <v>0</v>
+      </c>
       <c r="P43" s="14"/>
       <c r="Q43" s="17" t="str">
         <f>IF(LEN(TRIM(B43))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B43),FIND(" ",TRIM(B43)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B43),FIND(" ",TRIM(B43)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="44" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="15"/>
-      <c r="J44" s="16"/>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="16"/>
-      <c r="O44" s="19"/>
+      <c r="A44" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="D44" s="15">
+        <v>0</v>
+      </c>
+      <c r="E44" s="15">
+        <v>0</v>
+      </c>
+      <c r="F44" s="15">
+        <v>0</v>
+      </c>
+      <c r="G44" s="15">
+        <v>0</v>
+      </c>
+      <c r="H44" s="15">
+        <v>1</v>
+      </c>
+      <c r="I44" s="15">
+        <v>0</v>
+      </c>
+      <c r="J44" s="16">
+        <v>0</v>
+      </c>
+      <c r="K44" s="16">
+        <v>1</v>
+      </c>
+      <c r="L44" s="16">
+        <v>0</v>
+      </c>
+      <c r="M44" s="16">
+        <v>0</v>
+      </c>
+      <c r="N44" s="16">
+        <v>0</v>
+      </c>
+      <c r="O44" s="19">
+        <v>0</v>
+      </c>
       <c r="P44" s="14"/>
       <c r="Q44" s="17" t="str">
         <f>IF(LEN(TRIM(B44))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B44),FIND(" ",TRIM(B44)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B44),FIND(" ",TRIM(B44)&amp;" ")-1)))</f>
-        <v/>
+        <v>경기</v>
       </c>
     </row>
     <row r="45" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A45" s="14"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15"/>
-      <c r="J45" s="16"/>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="16"/>
-      <c r="O45" s="19"/>
+      <c r="A45" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D45" s="15">
+        <v>0</v>
+      </c>
+      <c r="E45" s="15">
+        <v>0</v>
+      </c>
+      <c r="F45" s="15">
+        <v>0</v>
+      </c>
+      <c r="G45" s="15">
+        <v>0</v>
+      </c>
+      <c r="H45" s="15">
+        <v>1</v>
+      </c>
+      <c r="I45" s="15">
+        <v>0</v>
+      </c>
+      <c r="J45" s="16">
+        <v>1</v>
+      </c>
+      <c r="K45" s="16">
+        <v>1</v>
+      </c>
+      <c r="L45" s="16">
+        <v>0</v>
+      </c>
+      <c r="M45" s="16">
+        <v>0</v>
+      </c>
+      <c r="N45" s="16">
+        <v>0</v>
+      </c>
+      <c r="O45" s="19">
+        <v>0</v>
+      </c>
       <c r="P45" s="14"/>
       <c r="Q45" s="17" t="str">
         <f>IF(LEN(TRIM(B45))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B45),FIND(" ",TRIM(B45)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B45),FIND(" ",TRIM(B45)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="46" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A46" s="14"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15"/>
-      <c r="J46" s="16"/>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="16"/>
-      <c r="O46" s="19"/>
+      <c r="A46" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="B46" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="D46" s="15">
+        <v>0</v>
+      </c>
+      <c r="E46" s="15">
+        <v>1</v>
+      </c>
+      <c r="F46" s="15">
+        <v>0</v>
+      </c>
+      <c r="G46" s="15">
+        <v>0</v>
+      </c>
+      <c r="H46" s="15">
+        <v>0</v>
+      </c>
+      <c r="I46" s="15">
+        <v>0</v>
+      </c>
+      <c r="J46" s="16">
+        <v>1</v>
+      </c>
+      <c r="K46" s="16">
+        <v>1</v>
+      </c>
+      <c r="L46" s="16">
+        <v>1</v>
+      </c>
+      <c r="M46" s="16">
+        <v>0</v>
+      </c>
+      <c r="N46" s="16">
+        <v>0</v>
+      </c>
+      <c r="O46" s="19">
+        <v>0</v>
+      </c>
       <c r="P46" s="14"/>
       <c r="Q46" s="17" t="str">
         <f>IF(LEN(TRIM(B46))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B46),FIND(" ",TRIM(B46)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B46),FIND(" ",TRIM(B46)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="47" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A47" s="14"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="16"/>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="16"/>
-      <c r="O47" s="19"/>
+      <c r="A47" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="D47" s="15">
+        <v>0</v>
+      </c>
+      <c r="E47" s="15">
+        <v>0</v>
+      </c>
+      <c r="F47" s="15">
+        <v>0</v>
+      </c>
+      <c r="G47" s="15">
+        <v>1</v>
+      </c>
+      <c r="H47" s="15">
+        <v>0</v>
+      </c>
+      <c r="I47" s="15">
+        <v>0</v>
+      </c>
+      <c r="J47" s="16">
+        <v>1</v>
+      </c>
+      <c r="K47" s="16">
+        <v>1</v>
+      </c>
+      <c r="L47" s="16">
+        <v>0</v>
+      </c>
+      <c r="M47" s="16">
+        <v>0</v>
+      </c>
+      <c r="N47" s="16">
+        <v>0</v>
+      </c>
+      <c r="O47" s="19">
+        <v>0</v>
+      </c>
       <c r="P47" s="14"/>
       <c r="Q47" s="17" t="str">
         <f>IF(LEN(TRIM(B47))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B47),FIND(" ",TRIM(B47)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B47),FIND(" ",TRIM(B47)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="48" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A48" s="14"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="15"/>
-      <c r="I48" s="15"/>
-      <c r="J48" s="16"/>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="16"/>
-      <c r="O48" s="19"/>
-      <c r="P48" s="14"/>
+      <c r="A48" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="D48" s="15">
+        <v>0</v>
+      </c>
+      <c r="E48" s="15">
+        <v>0</v>
+      </c>
+      <c r="F48" s="15">
+        <v>0</v>
+      </c>
+      <c r="G48" s="15">
+        <v>1</v>
+      </c>
+      <c r="H48" s="15">
+        <v>0</v>
+      </c>
+      <c r="I48" s="15">
+        <v>0</v>
+      </c>
+      <c r="J48" s="16">
+        <v>1</v>
+      </c>
+      <c r="K48" s="16">
+        <v>0</v>
+      </c>
+      <c r="L48" s="16">
+        <v>1</v>
+      </c>
+      <c r="M48" s="16">
+        <v>0</v>
+      </c>
+      <c r="N48" s="16">
+        <v>0</v>
+      </c>
+      <c r="O48" s="19">
+        <v>0</v>
+      </c>
+      <c r="P48" s="14" t="s">
+        <v>241</v>
+      </c>
       <c r="Q48" s="17" t="str">
         <f>IF(LEN(TRIM(B48))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B48),FIND(" ",TRIM(B48)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B48),FIND(" ",TRIM(B48)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="49" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A49" s="14"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="15"/>
-      <c r="F49" s="15"/>
-      <c r="G49" s="15"/>
-      <c r="H49" s="15"/>
-      <c r="I49" s="15"/>
-      <c r="J49" s="16"/>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="16"/>
-      <c r="O49" s="19"/>
+      <c r="A49" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="D49" s="15">
+        <v>0</v>
+      </c>
+      <c r="E49" s="15">
+        <v>0</v>
+      </c>
+      <c r="F49" s="15">
+        <v>0</v>
+      </c>
+      <c r="G49" s="15">
+        <v>1</v>
+      </c>
+      <c r="H49" s="15">
+        <v>0</v>
+      </c>
+      <c r="I49" s="15">
+        <v>0</v>
+      </c>
+      <c r="J49" s="16">
+        <v>0</v>
+      </c>
+      <c r="K49" s="16">
+        <v>1</v>
+      </c>
+      <c r="L49" s="16">
+        <v>0</v>
+      </c>
+      <c r="M49" s="16">
+        <v>0</v>
+      </c>
+      <c r="N49" s="16">
+        <v>0</v>
+      </c>
+      <c r="O49" s="19">
+        <v>0</v>
+      </c>
       <c r="P49" s="14"/>
       <c r="Q49" s="17" t="str">
         <f>IF(LEN(TRIM(B49))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B49),FIND(" ",TRIM(B49)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B49),FIND(" ",TRIM(B49)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="50" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A50" s="14"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
-      <c r="F50" s="15"/>
-      <c r="G50" s="15"/>
-      <c r="H50" s="15"/>
-      <c r="I50" s="15"/>
-      <c r="J50" s="16"/>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="16"/>
-      <c r="O50" s="19"/>
+      <c r="A50" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="D50" s="15">
+        <v>0</v>
+      </c>
+      <c r="E50" s="15">
+        <v>0</v>
+      </c>
+      <c r="F50" s="15">
+        <v>0</v>
+      </c>
+      <c r="G50" s="15">
+        <v>1</v>
+      </c>
+      <c r="H50" s="15">
+        <v>0</v>
+      </c>
+      <c r="I50" s="15">
+        <v>0</v>
+      </c>
+      <c r="J50" s="16">
+        <v>1</v>
+      </c>
+      <c r="K50" s="16">
+        <v>1</v>
+      </c>
+      <c r="L50" s="16">
+        <v>0</v>
+      </c>
+      <c r="M50" s="16">
+        <v>0</v>
+      </c>
+      <c r="N50" s="16">
+        <v>0</v>
+      </c>
+      <c r="O50" s="19">
+        <v>0</v>
+      </c>
       <c r="P50" s="14"/>
       <c r="Q50" s="17" t="str">
         <f>IF(LEN(TRIM(B50))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B50),FIND(" ",TRIM(B50)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B50),FIND(" ",TRIM(B50)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="51" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A51" s="14"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="15"/>
-      <c r="F51" s="15"/>
-      <c r="G51" s="15"/>
-      <c r="H51" s="15"/>
-      <c r="I51" s="15"/>
-      <c r="J51" s="16"/>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="16"/>
-      <c r="O51" s="19"/>
-      <c r="P51" s="14"/>
+      <c r="A51" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="D51" s="15">
+        <v>0</v>
+      </c>
+      <c r="E51" s="15">
+        <v>0</v>
+      </c>
+      <c r="F51" s="15">
+        <v>0</v>
+      </c>
+      <c r="G51" s="15">
+        <v>0</v>
+      </c>
+      <c r="H51" s="15">
+        <v>1</v>
+      </c>
+      <c r="I51" s="15">
+        <v>0</v>
+      </c>
+      <c r="J51" s="16">
+        <v>1</v>
+      </c>
+      <c r="K51" s="16">
+        <v>1</v>
+      </c>
+      <c r="L51" s="16">
+        <v>0</v>
+      </c>
+      <c r="M51" s="16">
+        <v>0</v>
+      </c>
+      <c r="N51" s="16">
+        <v>0</v>
+      </c>
+      <c r="O51" s="19">
+        <v>0</v>
+      </c>
+      <c r="P51" s="14" t="s">
+        <v>248</v>
+      </c>
       <c r="Q51" s="17" t="str">
         <f>IF(LEN(TRIM(B51))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B51),FIND(" ",TRIM(B51)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B51),FIND(" ",TRIM(B51)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="52" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A52" s="14"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="15"/>
-      <c r="E52" s="15"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
-      <c r="H52" s="15"/>
-      <c r="I52" s="15"/>
-      <c r="J52" s="16"/>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="16"/>
-      <c r="O52" s="19"/>
+      <c r="A52" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="B52" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="D52" s="15">
+        <v>0</v>
+      </c>
+      <c r="E52" s="15">
+        <v>1</v>
+      </c>
+      <c r="F52" s="15">
+        <v>0</v>
+      </c>
+      <c r="G52" s="15">
+        <v>0</v>
+      </c>
+      <c r="H52" s="15">
+        <v>0</v>
+      </c>
+      <c r="I52" s="15">
+        <v>0</v>
+      </c>
+      <c r="J52" s="16">
+        <v>0</v>
+      </c>
+      <c r="K52" s="16">
+        <v>1</v>
+      </c>
+      <c r="L52" s="16">
+        <v>1</v>
+      </c>
+      <c r="M52" s="16">
+        <v>0</v>
+      </c>
+      <c r="N52" s="16">
+        <v>0</v>
+      </c>
+      <c r="O52" s="19">
+        <v>0</v>
+      </c>
       <c r="P52" s="14"/>
       <c r="Q52" s="17" t="str">
         <f>IF(LEN(TRIM(B52))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B52),FIND(" ",TRIM(B52)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B52),FIND(" ",TRIM(B52)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="53" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A53" s="14"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="15"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="16"/>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="16"/>
-      <c r="O53" s="19"/>
-      <c r="P53" s="14"/>
+      <c r="A53" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="D53" s="15">
+        <v>0</v>
+      </c>
+      <c r="E53" s="15">
+        <v>0</v>
+      </c>
+      <c r="F53" s="15">
+        <v>0</v>
+      </c>
+      <c r="G53" s="15">
+        <v>0</v>
+      </c>
+      <c r="H53" s="15">
+        <v>1</v>
+      </c>
+      <c r="I53" s="15">
+        <v>0</v>
+      </c>
+      <c r="J53" s="16">
+        <v>1</v>
+      </c>
+      <c r="K53" s="16">
+        <v>1</v>
+      </c>
+      <c r="L53" s="16">
+        <v>0</v>
+      </c>
+      <c r="M53" s="16">
+        <v>0</v>
+      </c>
+      <c r="N53" s="16">
+        <v>0</v>
+      </c>
+      <c r="O53" s="19">
+        <v>0</v>
+      </c>
+      <c r="P53" s="14" t="s">
+        <v>262</v>
+      </c>
       <c r="Q53" s="17" t="str">
         <f>IF(LEN(TRIM(B53))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B53),FIND(" ",TRIM(B53)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B53),FIND(" ",TRIM(B53)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="54" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A54" s="14"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15"/>
-      <c r="J54" s="16"/>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="16"/>
-      <c r="O54" s="19"/>
-      <c r="P54" s="14"/>
+      <c r="A54" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="B54" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="C54" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="D54" s="15">
+        <v>0</v>
+      </c>
+      <c r="E54" s="15">
+        <v>0</v>
+      </c>
+      <c r="F54" s="15">
+        <v>0</v>
+      </c>
+      <c r="G54" s="15">
+        <v>1</v>
+      </c>
+      <c r="H54" s="15">
+        <v>1</v>
+      </c>
+      <c r="I54" s="15">
+        <v>0</v>
+      </c>
+      <c r="J54" s="16">
+        <v>1</v>
+      </c>
+      <c r="K54" s="16">
+        <v>1</v>
+      </c>
+      <c r="L54" s="16">
+        <v>1</v>
+      </c>
+      <c r="M54" s="16">
+        <v>0</v>
+      </c>
+      <c r="N54" s="16">
+        <v>0</v>
+      </c>
+      <c r="O54" s="19">
+        <v>0</v>
+      </c>
+      <c r="P54" s="14" t="s">
+        <v>261</v>
+      </c>
       <c r="Q54" s="17" t="str">
         <f>IF(LEN(TRIM(B54))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B54),FIND(" ",TRIM(B54)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B54),FIND(" ",TRIM(B54)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="55" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A55" s="14"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="15"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
-      <c r="H55" s="15"/>
-      <c r="I55" s="15"/>
-      <c r="J55" s="16"/>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
-      <c r="N55" s="16"/>
-      <c r="O55" s="19"/>
-      <c r="P55" s="14"/>
+      <c r="A55" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="C55" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="D55" s="15">
+        <v>0</v>
+      </c>
+      <c r="E55" s="15">
+        <v>1</v>
+      </c>
+      <c r="F55" s="15">
+        <v>0</v>
+      </c>
+      <c r="G55" s="15">
+        <v>0</v>
+      </c>
+      <c r="H55" s="15">
+        <v>0</v>
+      </c>
+      <c r="I55" s="15">
+        <v>0</v>
+      </c>
+      <c r="J55" s="16">
+        <v>0</v>
+      </c>
+      <c r="K55" s="16">
+        <v>0</v>
+      </c>
+      <c r="L55" s="16">
+        <v>1</v>
+      </c>
+      <c r="M55" s="16">
+        <v>0</v>
+      </c>
+      <c r="N55" s="16">
+        <v>0</v>
+      </c>
+      <c r="O55" s="19">
+        <v>0</v>
+      </c>
+      <c r="P55" s="14" t="s">
+        <v>266</v>
+      </c>
       <c r="Q55" s="17" t="str">
         <f>IF(LEN(TRIM(B55))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B55),FIND(" ",TRIM(B55)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B55),FIND(" ",TRIM(B55)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="56" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A56" s="14"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="15"/>
-      <c r="I56" s="15"/>
-      <c r="J56" s="16"/>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
-      <c r="N56" s="16"/>
-      <c r="O56" s="19"/>
-      <c r="P56" s="14"/>
+      <c r="A56" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B56" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="C56" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="D56" s="15">
+        <v>0</v>
+      </c>
+      <c r="E56" s="15">
+        <v>0</v>
+      </c>
+      <c r="F56" s="15">
+        <v>0</v>
+      </c>
+      <c r="G56" s="15">
+        <v>0</v>
+      </c>
+      <c r="H56" s="15">
+        <v>1</v>
+      </c>
+      <c r="I56" s="15">
+        <v>0</v>
+      </c>
+      <c r="J56" s="16">
+        <v>1</v>
+      </c>
+      <c r="K56" s="16">
+        <v>1</v>
+      </c>
+      <c r="L56" s="16">
+        <v>0</v>
+      </c>
+      <c r="M56" s="16">
+        <v>0</v>
+      </c>
+      <c r="N56" s="16">
+        <v>0</v>
+      </c>
+      <c r="O56" s="19">
+        <v>0</v>
+      </c>
+      <c r="P56" s="14" t="s">
+        <v>273</v>
+      </c>
       <c r="Q56" s="17" t="str">
         <f>IF(LEN(TRIM(B56))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B56),FIND(" ",TRIM(B56)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B56),FIND(" ",TRIM(B56)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="57" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A57" s="14"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="15"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="15"/>
-      <c r="J57" s="16"/>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
-      <c r="M57" s="16"/>
-      <c r="N57" s="16"/>
-      <c r="O57" s="19"/>
+      <c r="A57" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="B57" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="C57" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="D57" s="15">
+        <v>0</v>
+      </c>
+      <c r="E57" s="15">
+        <v>0</v>
+      </c>
+      <c r="F57" s="15">
+        <v>0</v>
+      </c>
+      <c r="G57" s="15">
+        <v>1</v>
+      </c>
+      <c r="H57" s="15">
+        <v>1</v>
+      </c>
+      <c r="I57" s="15">
+        <v>0</v>
+      </c>
+      <c r="J57" s="16">
+        <v>1</v>
+      </c>
+      <c r="K57" s="16">
+        <v>1</v>
+      </c>
+      <c r="L57" s="16">
+        <v>0</v>
+      </c>
+      <c r="M57" s="16">
+        <v>0</v>
+      </c>
+      <c r="N57" s="16">
+        <v>0</v>
+      </c>
+      <c r="O57" s="19">
+        <v>0</v>
+      </c>
       <c r="P57" s="14"/>
       <c r="Q57" s="17" t="str">
         <f>IF(LEN(TRIM(B57))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B57),FIND(" ",TRIM(B57)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B57),FIND(" ",TRIM(B57)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="58" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A58" s="14"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="15"/>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
-      <c r="H58" s="15"/>
-      <c r="I58" s="15"/>
-      <c r="J58" s="16"/>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
-      <c r="N58" s="16"/>
-      <c r="O58" s="19"/>
-      <c r="P58" s="14"/>
+      <c r="A58" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="B58" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="C58" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="D58" s="15">
+        <v>0</v>
+      </c>
+      <c r="E58" s="15">
+        <v>0</v>
+      </c>
+      <c r="F58" s="15">
+        <v>0</v>
+      </c>
+      <c r="G58" s="15">
+        <v>0</v>
+      </c>
+      <c r="H58" s="15">
+        <v>1</v>
+      </c>
+      <c r="I58" s="15">
+        <v>0</v>
+      </c>
+      <c r="J58" s="16">
+        <v>1</v>
+      </c>
+      <c r="K58" s="16">
+        <v>1</v>
+      </c>
+      <c r="L58" s="16">
+        <v>1</v>
+      </c>
+      <c r="M58" s="16">
+        <v>0</v>
+      </c>
+      <c r="N58" s="16">
+        <v>0</v>
+      </c>
+      <c r="O58" s="19">
+        <v>0</v>
+      </c>
+      <c r="P58" s="14" t="s">
+        <v>274</v>
+      </c>
       <c r="Q58" s="17" t="str">
         <f>IF(LEN(TRIM(B58))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B58),FIND(" ",TRIM(B58)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B58),FIND(" ",TRIM(B58)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="59" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A59" s="14"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="15"/>
-      <c r="I59" s="15"/>
-      <c r="J59" s="16"/>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
-      <c r="N59" s="16"/>
-      <c r="O59" s="19"/>
-      <c r="P59" s="14"/>
+      <c r="A59" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="B59" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="C59" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="D59" s="15">
+        <v>0</v>
+      </c>
+      <c r="E59" s="15">
+        <v>0</v>
+      </c>
+      <c r="F59" s="15">
+        <v>0</v>
+      </c>
+      <c r="G59" s="15">
+        <v>0</v>
+      </c>
+      <c r="H59" s="15">
+        <v>1</v>
+      </c>
+      <c r="I59" s="15">
+        <v>0</v>
+      </c>
+      <c r="J59" s="16">
+        <v>1</v>
+      </c>
+      <c r="K59" s="16">
+        <v>0</v>
+      </c>
+      <c r="L59" s="16">
+        <v>1</v>
+      </c>
+      <c r="M59" s="16">
+        <v>0</v>
+      </c>
+      <c r="N59" s="16">
+        <v>0</v>
+      </c>
+      <c r="O59" s="19">
+        <v>0</v>
+      </c>
+      <c r="P59" s="14" t="s">
+        <v>278</v>
+      </c>
       <c r="Q59" s="17" t="str">
         <f>IF(LEN(TRIM(B59))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B59),FIND(" ",TRIM(B59)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B59),FIND(" ",TRIM(B59)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="60" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A60" s="14"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
-      <c r="H60" s="15"/>
-      <c r="I60" s="15"/>
-      <c r="J60" s="16"/>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="16"/>
-      <c r="O60" s="19"/>
-      <c r="P60" s="14"/>
+      <c r="A60" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="C60" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="D60" s="15">
+        <v>0</v>
+      </c>
+      <c r="E60" s="15">
+        <v>0</v>
+      </c>
+      <c r="F60" s="15">
+        <v>0</v>
+      </c>
+      <c r="G60" s="15">
+        <v>0</v>
+      </c>
+      <c r="H60" s="15">
+        <v>1</v>
+      </c>
+      <c r="I60" s="15">
+        <v>0</v>
+      </c>
+      <c r="J60" s="16">
+        <v>1</v>
+      </c>
+      <c r="K60" s="16">
+        <v>1</v>
+      </c>
+      <c r="L60" s="16">
+        <v>0</v>
+      </c>
+      <c r="M60" s="16">
+        <v>0</v>
+      </c>
+      <c r="N60" s="16">
+        <v>0</v>
+      </c>
+      <c r="O60" s="19">
+        <v>0</v>
+      </c>
+      <c r="P60" s="14" t="s">
+        <v>282</v>
+      </c>
       <c r="Q60" s="17" t="str">
         <f>IF(LEN(TRIM(B60))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B60),FIND(" ",TRIM(B60)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B60),FIND(" ",TRIM(B60)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="61" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A61" s="14"/>
-      <c r="B61" s="14"/>
-      <c r="C61" s="14"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="16"/>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-      <c r="N61" s="16"/>
-      <c r="O61" s="19"/>
-      <c r="P61" s="14"/>
+      <c r="A61" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="B61" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="C61" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="D61" s="15">
+        <v>0</v>
+      </c>
+      <c r="E61" s="15">
+        <v>0</v>
+      </c>
+      <c r="F61" s="15">
+        <v>0</v>
+      </c>
+      <c r="G61" s="15">
+        <v>1</v>
+      </c>
+      <c r="H61" s="15">
+        <v>0</v>
+      </c>
+      <c r="I61" s="15">
+        <v>0</v>
+      </c>
+      <c r="J61" s="16">
+        <v>0</v>
+      </c>
+      <c r="K61" s="16">
+        <v>0</v>
+      </c>
+      <c r="L61" s="16">
+        <v>1</v>
+      </c>
+      <c r="M61" s="16">
+        <v>0</v>
+      </c>
+      <c r="N61" s="16">
+        <v>0</v>
+      </c>
+      <c r="O61" s="19">
+        <v>0</v>
+      </c>
+      <c r="P61" s="14" t="s">
+        <v>286</v>
+      </c>
       <c r="Q61" s="17" t="str">
         <f>IF(LEN(TRIM(B61))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B61),FIND(" ",TRIM(B61)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B61),FIND(" ",TRIM(B61)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="62" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A62" s="14"/>
-      <c r="B62" s="14"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="15"/>
-      <c r="G62" s="15"/>
-      <c r="H62" s="15"/>
-      <c r="I62" s="15"/>
-      <c r="J62" s="16"/>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="16"/>
-      <c r="O62" s="19"/>
-      <c r="P62" s="14"/>
+      <c r="A62" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="B62" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="C62" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="D62" s="15">
+        <v>0</v>
+      </c>
+      <c r="E62" s="15">
+        <v>0</v>
+      </c>
+      <c r="F62" s="15">
+        <v>0</v>
+      </c>
+      <c r="G62" s="15">
+        <v>1</v>
+      </c>
+      <c r="H62" s="15">
+        <v>0</v>
+      </c>
+      <c r="I62" s="15">
+        <v>0</v>
+      </c>
+      <c r="J62" s="16">
+        <v>0</v>
+      </c>
+      <c r="K62" s="16">
+        <v>0</v>
+      </c>
+      <c r="L62" s="16">
+        <v>1</v>
+      </c>
+      <c r="M62" s="16">
+        <v>0</v>
+      </c>
+      <c r="N62" s="16">
+        <v>0</v>
+      </c>
+      <c r="O62" s="19">
+        <v>0</v>
+      </c>
+      <c r="P62" s="14" t="s">
+        <v>286</v>
+      </c>
       <c r="Q62" s="17" t="str">
         <f>IF(LEN(TRIM(B62))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B62),FIND(" ",TRIM(B62)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B62),FIND(" ",TRIM(B62)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="63" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A63" s="14"/>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="15"/>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15"/>
-      <c r="H63" s="15"/>
-      <c r="I63" s="15"/>
-      <c r="J63" s="16"/>
-      <c r="K63" s="16"/>
-      <c r="L63" s="16"/>
-      <c r="M63" s="16"/>
-      <c r="N63" s="16"/>
-      <c r="O63" s="19"/>
+      <c r="A63" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="B63" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="C63" s="14" t="s">
+        <v>295</v>
+      </c>
+      <c r="D63" s="15">
+        <v>0</v>
+      </c>
+      <c r="E63" s="15">
+        <v>0</v>
+      </c>
+      <c r="F63" s="15">
+        <v>0</v>
+      </c>
+      <c r="G63" s="15">
+        <v>1</v>
+      </c>
+      <c r="H63" s="15">
+        <v>0</v>
+      </c>
+      <c r="I63" s="15">
+        <v>0</v>
+      </c>
+      <c r="J63" s="16">
+        <v>1</v>
+      </c>
+      <c r="K63" s="16">
+        <v>1</v>
+      </c>
+      <c r="L63" s="16">
+        <v>1</v>
+      </c>
+      <c r="M63" s="16">
+        <v>0</v>
+      </c>
+      <c r="N63" s="16">
+        <v>0</v>
+      </c>
+      <c r="O63" s="19">
+        <v>0</v>
+      </c>
       <c r="P63" s="14"/>
       <c r="Q63" s="17" t="str">
         <f>IF(LEN(TRIM(B63))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B63),FIND(" ",TRIM(B63)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B63),FIND(" ",TRIM(B63)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="64" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A64" s="14"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
-      <c r="D64" s="15"/>
-      <c r="E64" s="15"/>
-      <c r="F64" s="15"/>
-      <c r="G64" s="15"/>
-      <c r="H64" s="15"/>
-      <c r="I64" s="15"/>
-      <c r="J64" s="16"/>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-      <c r="N64" s="16"/>
-      <c r="O64" s="19"/>
+      <c r="A64" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="B64" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="C64" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="D64" s="15">
+        <v>0</v>
+      </c>
+      <c r="E64" s="15">
+        <v>0</v>
+      </c>
+      <c r="F64" s="15">
+        <v>0</v>
+      </c>
+      <c r="G64" s="15">
+        <v>0</v>
+      </c>
+      <c r="H64" s="15">
+        <v>1</v>
+      </c>
+      <c r="I64" s="15">
+        <v>0</v>
+      </c>
+      <c r="J64" s="16">
+        <v>0</v>
+      </c>
+      <c r="K64" s="16">
+        <v>1</v>
+      </c>
+      <c r="L64" s="16">
+        <v>0</v>
+      </c>
+      <c r="M64" s="16">
+        <v>0</v>
+      </c>
+      <c r="N64" s="16">
+        <v>0</v>
+      </c>
+      <c r="O64" s="19">
+        <v>0</v>
+      </c>
       <c r="P64" s="14"/>
       <c r="Q64" s="17" t="str">
         <f>IF(LEN(TRIM(B64))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B64),FIND(" ",TRIM(B64)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B64),FIND(" ",TRIM(B64)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="65" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A65" s="14"/>
-      <c r="B65" s="14"/>
-      <c r="C65" s="14"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="15"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
-      <c r="H65" s="15"/>
-      <c r="I65" s="15"/>
-      <c r="J65" s="16"/>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
-      <c r="N65" s="16"/>
-      <c r="O65" s="19"/>
-      <c r="P65" s="14"/>
+      <c r="A65" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="B65" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="D65" s="15">
+        <v>0</v>
+      </c>
+      <c r="E65" s="15">
+        <v>0</v>
+      </c>
+      <c r="F65" s="15">
+        <v>0</v>
+      </c>
+      <c r="G65" s="15">
+        <v>1</v>
+      </c>
+      <c r="H65" s="15">
+        <v>0</v>
+      </c>
+      <c r="I65" s="15">
+        <v>0</v>
+      </c>
+      <c r="J65" s="16">
+        <v>1</v>
+      </c>
+      <c r="K65" s="16">
+        <v>1</v>
+      </c>
+      <c r="L65" s="16">
+        <v>1</v>
+      </c>
+      <c r="M65" s="16">
+        <v>0</v>
+      </c>
+      <c r="N65" s="16">
+        <v>0</v>
+      </c>
+      <c r="O65" s="19">
+        <v>0</v>
+      </c>
+      <c r="P65" s="14" t="s">
+        <v>299</v>
+      </c>
       <c r="Q65" s="17" t="str">
         <f>IF(LEN(TRIM(B65))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B65),FIND(" ",TRIM(B65)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B65),FIND(" ",TRIM(B65)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="66" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A66" s="14"/>
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
-      <c r="H66" s="15"/>
-      <c r="I66" s="15"/>
-      <c r="J66" s="16"/>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
-      <c r="N66" s="16"/>
-      <c r="O66" s="19"/>
+      <c r="A66" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="B66" s="14" t="s">
+        <v>303</v>
+      </c>
+      <c r="C66" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="D66" s="15">
+        <v>0</v>
+      </c>
+      <c r="E66" s="15">
+        <v>1</v>
+      </c>
+      <c r="F66" s="15">
+        <v>0</v>
+      </c>
+      <c r="G66" s="15">
+        <v>0</v>
+      </c>
+      <c r="H66" s="15">
+        <v>0</v>
+      </c>
+      <c r="I66" s="15">
+        <v>0</v>
+      </c>
+      <c r="J66" s="16">
+        <v>1</v>
+      </c>
+      <c r="K66" s="16">
+        <v>1</v>
+      </c>
+      <c r="L66" s="16">
+        <v>1</v>
+      </c>
+      <c r="M66" s="16">
+        <v>0</v>
+      </c>
+      <c r="N66" s="16">
+        <v>0</v>
+      </c>
+      <c r="O66" s="19">
+        <v>0</v>
+      </c>
       <c r="P66" s="14"/>
       <c r="Q66" s="17" t="str">
         <f>IF(LEN(TRIM(B66))=0,"",IFERROR(VLOOKUP(LEFT(TRIM(B66),FIND(" ",TRIM(B66)&amp;" ")-1),작성안내!$D$4:$E$23,2,FALSE),LEFT(TRIM(B66),FIND(" ",TRIM(B66)&amp;" ")-1)))</f>
-        <v/>
+        <v>서울</v>
       </c>
     </row>
     <row r="67" spans="1:17" ht="25.5" customHeight="1">

</xml_diff>